<commit_message>
fix(karaba): 말소신청서 수임자 번호 교체 (jin 2026-09-10)
karaba 「1.차량말소신청서」 C39 — 11-95-278048-01 → 731110-1041111.

- 그 칸은 **흰칸 + 매핑 없음**이라 양식에 박힌 값이 그대로 인쇄된다(SKILLS §8 #71).
  ⇒ 파일을 고치는 것 말고는 바꿀 방법이 없다.
- 3 세트 전수 검색 결과 **이 한 곳뿐**이다. system·heyman 은 수임자 영역이 공란이라
  (손으로 쓰는 칸) 영향 없다 — karaba 만 수임자를 고정으로 박아 쓴다.
- ⚠️ 라벨은 「사업자번호」인데 값은 주민등록번호 형식이다 — 별지17호 법정 서식이라 라벨을
  못 바꾸고, 수임자가 개인이라 그 칸에 개인 번호가 들어간다. 구 값은 자동차매매업 등록번호 형식.
- 저장은 stripHyperlinks(프로젝트 방식) + setPreCalculateFormulas(false).
  ⚠️ 셀 단위 setHyperlink(null) 로는 writer 가 "Invalid parameters" 로 죽는다 —
     시트의 getHyperlinkCollection() 을 돌아야 한다(DocumentFiller 와 같은 방식).

가드 = KarabaDeregistrationApplicationTest — 09-04 에 만든 그 테스트가 옛 값을 못박고 있어
**의도대로 빨갛게 잡았다**. 목적(수임자 값이 clearYellowFill 에 지워지지 않는지)은 그대로 두고
값만 갱신했다. 생성물의 셀을 실제로 읽으므로 양식이 깨졌으면 여기서 드러난다.

관련 14 pass.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZGn77LtEQCZsa35EZhs9x
</commit_message>
<xml_diff>
--- a/resources/templates/karaba/deregistration_application.xlsx
+++ b/resources/templates/karaba/deregistration_application.xlsx
@@ -295,7 +295,7 @@
     <t>길영채</t>
   </si>
   <si>
-    <t>11-95-278048-01</t>
+    <t>731110-1041111</t>
   </si>
 </sst>
 </file>
@@ -486,7 +486,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -505,9 +505,6 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="none"/>
-    </fill>
   </fills>
   <borders count="63">
     <border>
@@ -1630,10 +1627,10 @@
     <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="60" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="9" numFmtId="0" fillId="4" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="9" numFmtId="0" fillId="0" borderId="5" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
-    <xf xfId="0" fontId="9" numFmtId="166" fillId="4" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf xfId="0" fontId="9" numFmtId="166" fillId="0" borderId="5" applyFont="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" shrinkToFit="false"/>
     </xf>
   </cellXfs>

</xml_diff>